<commit_message>
Add test cases for login lockout (feat/login-lockout)
Test cases for G2 "Khoá đăng nhập": 5 wrong passwords in a row lock
sign-in for 15 minutes, for both staff and customers.

- TestCase_2_KhoaDangNhap.docx: 11 test cases covering the warning
  before the lock, the lock itself, the right password still refused
  while locked, unlocking by admin reset or OTP password reset, and
  phone layout; with screenshots
- TestCase_SEVEN11.xlsx: new sheet 2-KhoaDangNhap, summary updated
- 10 Pass (run in a real browser with Playwright on 21/10/2026),
  1 left for manual testing (TC-KDN-08, the lock expires after 15 min)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/dotnet/docs/test-cases/TestCase_SEVEN11.xlsx
+++ b/apps/dotnet/docs/test-cases/TestCase_SEVEN11.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1-DoiMatKhau" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2-KhoaDangNhap" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -510,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -617,31 +618,68 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>2-KhoaDangNhap</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Khoá đăng nhập sau 5 lần sai mật khẩu</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>feat/login-lockout</t>
+        </is>
+      </c>
+      <c r="D6" s="4">
+        <f>COUNTA('2-KhoaDangNhap'!A5:A15)</f>
+        <v/>
+      </c>
+      <c r="E6" s="4">
+        <f>COUNTIF('2-KhoaDangNhap'!H5:H15,"Pass")</f>
+        <v/>
+      </c>
+      <c r="F6" s="4">
+        <f>COUNTIF('2-KhoaDangNhap'!H5:H15,"Fail")</f>
+        <v/>
+      </c>
+      <c r="G6" s="4">
+        <f>D6-E6-F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="5">
+        <f>IF(D6=0,0,E6/D6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Tổng</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6">
-        <f>SUM(D5:D5)</f>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6">
+        <f>SUM(D5:D6)</f>
         <v/>
       </c>
-      <c r="E6" s="6">
-        <f>SUM(E5:E5)</f>
+      <c r="E7" s="6">
+        <f>SUM(E5:E6)</f>
         <v/>
       </c>
-      <c r="F6" s="6">
-        <f>SUM(F5:F5)</f>
+      <c r="F7" s="6">
+        <f>SUM(F5:F6)</f>
         <v/>
       </c>
-      <c r="G6" s="6">
-        <f>SUM(G5:G5)</f>
+      <c r="G7" s="6">
+        <f>SUM(G5:G6)</f>
         <v/>
       </c>
-      <c r="H6" s="7">
-        <f>IF(D6=0,0,E6/D6)</f>
+      <c r="H7" s="7">
+        <f>IF(D7=0,0,E7/D7)</f>
         <v/>
       </c>
     </row>
@@ -1571,4 +1609,656 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Khoá đăng nhập sau 5 lần sai mật khẩu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Nhánh: feat/login-lockout · App .NET: http://localhost:5711 · Tài khoản demo mật khẩu 123456</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Mã TC</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Mục đích kiểm thử</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Điều kiện trước</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Các bước</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Dữ liệu test</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Kết quả mong đợi</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Kết quả thực tế</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Ngày test</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>TC-KDN-01</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Sai mật khẩu lần đầu</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Có tài khoản nhân viên</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập với mật khẩu sai</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Mật khẩu: sai-1</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>Báo "Mật khẩu không đúng"</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>Đã chạy tự động bằng Playwright</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>TC-KDN-02</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Cảnh báo số lần thử còn lại</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Đã sai 3 lần liên tiếp</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập sai lần thứ 4</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Mật khẩu: sai-4</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Báo "Mật khẩu không đúng, còn 1 lần thử trước khi bị khoá 15 phút"</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>Đã chạy tự động bằng Playwright</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>TC-KDN-03</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Sai lần thứ 5 thì bị khoá</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Đã sai 4 lần liên tiếp</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập sai lần thứ 5</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Mật khẩu: sai-5</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>Báo "Đăng nhập tạm khoá do nhập sai mật khẩu 5 lần liên tiếp. Thử lại sau 15 phút."</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>Đã chạy tự động bằng Playwright</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>TC-KDN-04</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Đang khoá thì mật khẩu đúng cũng bị từ chối</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Tài khoản đang bị khoá (TC-KDN-03)</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>1. Đăng nhập bằng mật khẩu đúng</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Mật khẩu đúng</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Vẫn báo tạm khoá, không vào được</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>Đã chạy tự động bằng Playwright</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>TC-KDN-05</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Quản trị thấy nhân viên đang bị khoá</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Nhân viên đang bị khoá; đăng nhập admin@7eleven.demo / 123456</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>1. Mở hồ sơ nhân viên đó</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr"/>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Khung Mật khẩu hiện "Đăng nhập đang khoá tới HH:mm"</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>Đã chạy tự động bằng Playwright</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>TC-KDN-06</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Quản trị đặt lại mật khẩu thì mở khoá</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Như TC-KDN-05</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>1. Bấm Đặt lại mật khẩu
+2. Nhân viên đăng nhập bằng mật khẩu tạm</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr"/>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Hết cảnh báo khoá; nhân viên đăng nhập được ngay</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>Đã chạy tự động bằng Playwright</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>TC-KDN-07</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Đăng nhập đúng thì đếm lại từ đầu</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>quanly1006@7eleven.demo</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>1. Sai 4 lần liên tiếp
+2. Lần 5 nhập đúng
+3. Đăng xuất, nhập sai 1 lần</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr"/>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Bước 2 vào được; bước 3 chỉ báo "Mật khẩu không đúng", không bị khoá</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="J11" s="10" t="inlineStr">
+        <is>
+          <t>Đã chạy tự động bằng Playwright</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>TC-KDN-08</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Hết 15 phút thì tự mở khoá</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Tài khoản vừa bị khoá</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>1. Chờ 15 phút
+2. Đăng nhập bằng mật khẩu đúng</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr"/>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Đăng nhập được</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr"/>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>Chưa test</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="inlineStr"/>
+      <c r="J12" s="10" t="inlineStr">
+        <is>
+          <t>Tester chạy tay</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>TC-KDN-09</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Khách bị khoá sau 5 lần sai</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Khách 0987654321</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>1. Ở /dang-nhap nhập sai 5 lần
+2. Nhập mật khẩu đúng</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr"/>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Lần 3 báo còn 2 lần thử; lần 5 bị khoá; mật khẩu đúng vẫn bị từ chối</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="J13" s="10" t="inlineStr">
+        <is>
+          <t>Đã chạy tự động bằng Playwright</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>TC-KDN-10</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Khách mở khoá bằng Quên mật khẩu (OTP)</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Khách đang bị khoá</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>1. Bấm Quên mật khẩu, nhập số điện thoại
+2. Nhập mã OTP trong tin nhắn giả lập
+3. Đặt mật khẩu mới</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Mật khẩu mới: 123456</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Đăng nhập ngay; lần sau đăng nhập bình thường</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="J14" s="10" t="inlineStr">
+        <is>
+          <t>Đã chạy tự động bằng Playwright</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>TC-KDN-11</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Hiển thị trên điện thoại</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Trình duyệt ở chế độ điện thoại (390px)</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>1. Làm khách bị khoá như TC-KDN-09</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr"/>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Câu báo khoá hiện đủ dưới ô mật khẩu, không tràn ngang</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="10" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="J15" s="10" t="inlineStr">
+        <is>
+          <t>Đã chạy tự động bằng Playwright</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="H5:H15">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pass,Fail,Chưa test"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Record regression run for G1 and G2 on 22/10 (change-password, login-lockout)
Re-ran every existing test after merging main into dev:
- xUnit 92/92 pass
- Playwright walk-throughs for G1 "Đổi mật khẩu" and G2 "Khoá đăng nhập"
  pass (demo data reset first)
- Team e2e: admin-flows, pos-flow, storefront-pages pass; storefront-flow
  fails 1/74 on a hidden quick-add button on /khuyen-mai at phone width,
  which is already on main (storefront redesign), not caused by G1/G2

TestCase_SEVEN11.xlsx: G1/G2 rows now show the 22/10 run date; new sheet
"Hồi quy" logs each full re-run.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/dotnet/docs/test-cases/TestCase_SEVEN11.xlsx
+++ b/apps/dotnet/docs/test-cases/TestCase_SEVEN11.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1-DoiMatKhau" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2-KhoaDangNhap" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hồi quy" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1-DoiMatKhau" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2-KhoaDangNhap" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +57,18 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00067A36"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00B91C1C"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="4">
@@ -102,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -113,10 +126,16 @@
     <xf numFmtId="9" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -694,6 +713,218 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Nhật ký chạy lại toàn bộ test (hồi quy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Mỗi ngày chạy lại test của mọi chức năng đã làm, kèm bộ e2e của nhóm, để chắc code mới không làm hỏng code cũ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Ngày</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Lúc</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Bộ test</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Kết quả</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Sau khi làm G1, G2</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>xUnit</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>92/92 đạt</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Sau khi làm G1, G2</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Playwright G1, G2</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Sau khi làm G1, G2</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>e2e của nhóm (admin, pos, storefront-flow)</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>1 kiểm tra hỏng / 90</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>"logout toast" hỏng, có sẵn trên main; Phát đã sửa ngày 22/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Đầu ngày, sau khi gộp main</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>xUnit</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>92/92 đạt</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Đầu ngày, sau khi gộp main</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Playwright G1, G2</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Tạo lại dữ liệu mẫu trước khi chạy</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Đầu ngày, sau khi gộp main</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>e2e của nhóm (admin, pos, storefront-pages, storefront-flow)</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>1 kiểm tra hỏng / 74</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>storefront-flow: nút thêm nhanh ở /khuyen-mai bị ẩn trên điện thoại; có sẵn trên main (bản redesign), cần báo Phát</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -776,820 +1007,820 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>TC-DMK-01</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Nhân viên mới bị bắt đổi mật khẩu ở lần đăng nhập đầu</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Nhân viên mới do quản trị tạo (mật khẩu mặc định 123456)</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>1. Vào /Admin/Account/Login
 2. Nhập email nhân viên mới, mật khẩu 123456
 3. Bấm Đăng nhập</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Mật khẩu: 123456</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>Chuyển sang trang "Đặt mật khẩu mới", có dòng nhắc mật khẩu do người khác cấp</t>
         </is>
       </c>
-      <c r="G5" s="10" t="inlineStr">
+      <c r="G5" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H5" s="10" t="inlineStr">
+      <c r="H5" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I5" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J5" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>TC-DMK-02</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Chưa đổi mật khẩu thì không vào được trang quản lý</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Đang ở trang Đặt mật khẩu mới (TC-DMK-01)</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>1. Gõ thẳng địa chỉ /Admin/Pos</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr"/>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr"/>
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>Bị chuyển lại trang Đặt mật khẩu mới</t>
         </is>
       </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="G6" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="H6" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I6" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J6" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>TC-DMK-03</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Mật khẩu mới trùng mật khẩu hiện tại</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Đang ở trang đổi mật khẩu</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>1. Nhập mật khẩu hiện tại, mật khẩu mới, nhập lại giống nhau
 2. Bấm Lưu</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Hiện tại: 123456
 Mới: 123456
 Nhập lại: 123456</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Báo lỗi "Mật khẩu mới phải khác mật khẩu hiện tại"</t>
         </is>
       </c>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="G7" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="H7" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I7" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J7" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>TC-DMK-04</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Mật khẩu mới quá ngắn</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>Đang ở trang đổi mật khẩu</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>1. Nhập mật khẩu mới dưới 6 ký tự
 2. Bấm Lưu</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Mới: abc</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>Báo lỗi "Mật khẩu tối thiểu 6 ký tự"</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="G8" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="H8" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I8" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J8" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>TC-DMK-05</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Nhập lại mật khẩu không khớp</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Đang ở trang đổi mật khẩu</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>1. Nhập mật khẩu mới và nhập lại khác nhau
 2. Bấm Lưu</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>Mới: abcdef
 Nhập lại: abcdeg</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Báo lỗi "Mật khẩu nhập lại không khớp"</t>
         </is>
       </c>
-      <c r="G9" s="10" t="inlineStr">
+      <c r="G9" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="H9" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J9" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>TC-DMK-06</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Nhân viên mới đổi mật khẩu thành công</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Đang ở trang Đặt mật khẩu mới</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>1. Nhập đúng mật khẩu được cấp, mật khẩu mới hợp lệ, nhập lại khớp
 2. Bấm Lưu</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>Hiện tại: 123456
 Mới: thungan@2026</t>
         </is>
       </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>Thu ngân vào thẳng máy bán hàng (/Admin/Pos), hiện thông báo "Đã đổi mật khẩu"</t>
         </is>
       </c>
-      <c r="G10" s="10" t="inlineStr">
+      <c r="G10" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H10" s="10" t="inlineStr">
+      <c r="H10" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I10" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J10" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>TC-DMK-07</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Đổi mật khẩu từ menu, mật khẩu hiện tại sai</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Đăng nhập quanly1006@7eleven.demo</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>1. Bấm tên ở góc phải → Đổi mật khẩu
 2. Nhập sai mật khẩu hiện tại
 3. Bấm Lưu</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>Hiện tại: sai-mat-khau</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>Báo lỗi "Mật khẩu hiện tại không đúng"</t>
         </is>
       </c>
-      <c r="G11" s="10" t="inlineStr">
+      <c r="G11" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H11" s="10" t="inlineStr">
+      <c r="H11" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I11" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J11" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>TC-DMK-08</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Đổi mật khẩu từ menu thành công</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Đăng nhập quanly1006@7eleven.demo</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>1. Menu tài khoản → Đổi mật khẩu
 2. Nhập đúng mật khẩu hiện tại, mật khẩu mới hợp lệ
 3. Bấm Lưu</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>Mới: quanly@2026</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>Quay về trang đang xem, hiện "Đã đổi mật khẩu" (test xong đổi lại 123456)</t>
         </is>
       </c>
-      <c r="G12" s="10" t="inlineStr">
+      <c r="G12" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H12" s="10" t="inlineStr">
+      <c r="H12" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I12" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J12" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>TC-DMK-09</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Quản trị đặt lại mật khẩu nhân viên</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Đăng nhập admin@7eleven.demo / 123456</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>1. Nhân viên &amp; ca → mở hồ sơ một nhân viên
 2. Bấm Đặt lại mật khẩu → OK</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr"/>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr"/>
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>Thông báo hiện mật khẩu tạm 8 ký tự; khung Mật khẩu ghi "Đang dùng mật khẩu được cấp"</t>
         </is>
       </c>
-      <c r="G13" s="10" t="inlineStr">
+      <c r="G13" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H13" s="10" t="inlineStr">
+      <c r="H13" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I13" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J13" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>TC-DMK-10</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Mật khẩu cũ hết dùng được sau khi đặt lại</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Đã làm TC-DMK-09</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>1. Đăng nhập nhân viên đó bằng mật khẩu cũ</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>Mật khẩu cũ</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>Báo "Mật khẩu không đúng"</t>
         </is>
       </c>
-      <c r="G14" s="10" t="inlineStr">
+      <c r="G14" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H14" s="10" t="inlineStr">
+      <c r="H14" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I14" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J14" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J14" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>TC-DMK-11</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Đăng nhập bằng mật khẩu tạm bị bắt đổi</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Đã làm TC-DMK-09</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>1. Đăng nhập bằng mật khẩu tạm
 2. Đổi sang mật khẩu mới</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>Mật khẩu tạm ở TC-DMK-09</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>Bị chuyển sang trang Đặt mật khẩu mới; đổi xong vào được máy bán hàng</t>
         </is>
       </c>
-      <c r="G15" s="10" t="inlineStr">
+      <c r="G15" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H15" s="10" t="inlineStr">
+      <c r="H15" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I15" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J15" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>TC-DMK-12</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Quản lý cửa hàng không đặt lại được mật khẩu</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>Đăng nhập quanly1006@7eleven.demo</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>1. Nhân viên &amp; ca → mở hồ sơ một thu ngân</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr"/>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr"/>
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>Không có khung Mật khẩu, không có nút Đặt lại mật khẩu</t>
         </is>
       </c>
-      <c r="G16" s="10" t="inlineStr"/>
-      <c r="H16" s="10" t="inlineStr">
+      <c r="G16" s="12" t="inlineStr"/>
+      <c r="H16" s="12" t="inlineStr">
         <is>
           <t>Chưa test</t>
         </is>
       </c>
-      <c r="I16" s="10" t="inlineStr"/>
-      <c r="J16" s="10" t="inlineStr">
+      <c r="I16" s="12" t="inlineStr"/>
+      <c r="J16" s="12" t="inlineStr">
         <is>
           <t>Tester chạy tay</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>TC-DMK-13</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Quản trị không tự đặt lại mật khẩu của mình</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>Đăng nhập admin@7eleven.demo / 123456</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>1. Mở hồ sơ của chính mình (Nguyễn Minh Quân)</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr"/>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr"/>
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>Không có nút Đặt lại mật khẩu</t>
         </is>
       </c>
-      <c r="G17" s="10" t="inlineStr"/>
-      <c r="H17" s="10" t="inlineStr">
+      <c r="G17" s="12" t="inlineStr"/>
+      <c r="H17" s="12" t="inlineStr">
         <is>
           <t>Chưa test</t>
         </is>
       </c>
-      <c r="I17" s="10" t="inlineStr"/>
-      <c r="J17" s="10" t="inlineStr">
+      <c r="I17" s="12" t="inlineStr"/>
+      <c r="J17" s="12" t="inlineStr">
         <is>
           <t>Tester chạy tay</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>TC-DMK-14</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Khách đổi mật khẩu, nhập sai mật khẩu hiện tại</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>Khách đăng nhập 0901234567 / 123456</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>1. Tài khoản → tab Thông tin → khung Đổi mật khẩu
 2. Nhập sai mật khẩu hiện tại, nhập lại không khớp
 3. Bấm Đổi mật khẩu</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>Hiện tại: sai
 Mới: abcdef
 Nhập lại: abcdeg</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>Báo "Mật khẩu hiện tại không đúng" và "Mật khẩu nhập lại không khớp"</t>
         </is>
       </c>
-      <c r="G18" s="10" t="inlineStr">
+      <c r="G18" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H18" s="10" t="inlineStr">
+      <c r="H18" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I18" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J18" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I18" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>TC-DMK-15</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Khách đổi mật khẩu thành công</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Khách đăng nhập 0901234567 / 123456</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>1. Đổi sang mật khẩu mới
 2. Đăng xuất, đăng nhập bằng mật khẩu cũ
 3. Đăng nhập bằng mật khẩu mới</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>Mới: khach@2026</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>Hiện "Đã đổi mật khẩu"; mật khẩu cũ bị báo sai; mật khẩu mới đăng nhập được (test xong đổi lại 123456)</t>
         </is>
       </c>
-      <c r="G19" s="10" t="inlineStr">
+      <c r="G19" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H19" s="10" t="inlineStr">
+      <c r="H19" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I19" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J19" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J19" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>TC-DMK-16</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Hiển thị trên điện thoại</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>Trình duyệt ở chế độ điện thoại (390px)</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>1. Mở trang đổi mật khẩu nhân viên và tab Thông tin của khách</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr"/>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr"/>
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>Form hiển thị đủ, không tràn ngang</t>
         </is>
       </c>
-      <c r="G20" s="10" t="inlineStr">
+      <c r="G20" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H20" s="10" t="inlineStr">
+      <c r="H20" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I20" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J20" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J20" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1842,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1699,549 +1930,549 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>TC-KDN-01</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Sai mật khẩu lần đầu</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Có tài khoản nhân viên</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>1. Đăng nhập với mật khẩu sai</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Mật khẩu: sai-1</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>Báo "Mật khẩu không đúng"</t>
         </is>
       </c>
-      <c r="G5" s="10" t="inlineStr">
+      <c r="G5" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H5" s="10" t="inlineStr">
+      <c r="H5" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I5" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J5" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>TC-KDN-02</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Cảnh báo số lần thử còn lại</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Đã sai 3 lần liên tiếp</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>1. Đăng nhập sai lần thứ 4</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>Mật khẩu: sai-4</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>Báo "Mật khẩu không đúng, còn 1 lần thử trước khi bị khoá 15 phút"</t>
         </is>
       </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="G6" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="H6" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I6" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J6" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>TC-KDN-03</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Sai lần thứ 5 thì bị khoá</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Đã sai 4 lần liên tiếp</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>1. Đăng nhập sai lần thứ 5</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Mật khẩu: sai-5</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Báo "Đăng nhập tạm khoá do nhập sai mật khẩu 5 lần liên tiếp. Thử lại sau 15 phút."</t>
         </is>
       </c>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="G7" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr">
+      <c r="H7" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I7" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J7" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>TC-KDN-04</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Đang khoá thì mật khẩu đúng cũng bị từ chối</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>Tài khoản đang bị khoá (TC-KDN-03)</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>1. Đăng nhập bằng mật khẩu đúng</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Mật khẩu đúng</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>Vẫn báo tạm khoá, không vào được</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="G8" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="H8" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I8" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J8" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>TC-KDN-05</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Quản trị thấy nhân viên đang bị khoá</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Nhân viên đang bị khoá; đăng nhập admin@7eleven.demo / 123456</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>1. Mở hồ sơ nhân viên đó</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr"/>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr"/>
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Khung Mật khẩu hiện "Đăng nhập đang khoá tới HH:mm"</t>
         </is>
       </c>
-      <c r="G9" s="10" t="inlineStr">
+      <c r="G9" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="H9" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J9" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>TC-KDN-06</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Quản trị đặt lại mật khẩu thì mở khoá</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Như TC-KDN-05</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>1. Bấm Đặt lại mật khẩu
 2. Nhân viên đăng nhập bằng mật khẩu tạm</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr"/>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr"/>
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>Hết cảnh báo khoá; nhân viên đăng nhập được ngay</t>
         </is>
       </c>
-      <c r="G10" s="10" t="inlineStr">
+      <c r="G10" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H10" s="10" t="inlineStr">
+      <c r="H10" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I10" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J10" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>TC-KDN-07</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Đăng nhập đúng thì đếm lại từ đầu</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>quanly1006@7eleven.demo</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>1. Sai 4 lần liên tiếp
 2. Lần 5 nhập đúng
 3. Đăng xuất, nhập sai 1 lần</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr"/>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr"/>
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>Bước 2 vào được; bước 3 chỉ báo "Mật khẩu không đúng", không bị khoá</t>
         </is>
       </c>
-      <c r="G11" s="10" t="inlineStr">
+      <c r="G11" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H11" s="10" t="inlineStr">
+      <c r="H11" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I11" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J11" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>TC-KDN-08</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Hết 15 phút thì tự mở khoá</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Tài khoản vừa bị khoá</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>1. Chờ 15 phút
 2. Đăng nhập bằng mật khẩu đúng</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr"/>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr"/>
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>Đăng nhập được</t>
         </is>
       </c>
-      <c r="G12" s="10" t="inlineStr"/>
-      <c r="H12" s="10" t="inlineStr">
+      <c r="G12" s="12" t="inlineStr"/>
+      <c r="H12" s="12" t="inlineStr">
         <is>
           <t>Chưa test</t>
         </is>
       </c>
-      <c r="I12" s="10" t="inlineStr"/>
-      <c r="J12" s="10" t="inlineStr">
+      <c r="I12" s="12" t="inlineStr"/>
+      <c r="J12" s="12" t="inlineStr">
         <is>
           <t>Tester chạy tay</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>TC-KDN-09</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Khách bị khoá sau 5 lần sai</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Khách 0987654321</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>1. Ở /dang-nhap nhập sai 5 lần
 2. Nhập mật khẩu đúng</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr"/>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr"/>
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>Lần 3 báo còn 2 lần thử; lần 5 bị khoá; mật khẩu đúng vẫn bị từ chối</t>
         </is>
       </c>
-      <c r="G13" s="10" t="inlineStr">
+      <c r="G13" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H13" s="10" t="inlineStr">
+      <c r="H13" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I13" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J13" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>TC-KDN-10</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Khách mở khoá bằng Quên mật khẩu (OTP)</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Khách đang bị khoá</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>1. Bấm Quên mật khẩu, nhập số điện thoại
 2. Nhập mã OTP trong tin nhắn giả lập
 3. Đặt mật khẩu mới</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>Mật khẩu mới: 123456</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>Đăng nhập ngay; lần sau đăng nhập bình thường</t>
         </is>
       </c>
-      <c r="G14" s="10" t="inlineStr">
+      <c r="G14" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H14" s="10" t="inlineStr">
+      <c r="H14" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I14" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J14" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J14" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>TC-KDN-11</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Hiển thị trên điện thoại</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Trình duyệt ở chế độ điện thoại (390px)</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>1. Làm khách bị khoá như TC-KDN-09</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr"/>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr"/>
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>Câu báo khoá hiện đủ dưới ô mật khẩu, không tràn ngang</t>
         </is>
       </c>
-      <c r="G15" s="10" t="inlineStr">
+      <c r="G15" s="12" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H15" s="10" t="inlineStr">
+      <c r="H15" s="12" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="I15" s="10" t="inlineStr">
-        <is>
-          <t>21/10/2026</t>
-        </is>
-      </c>
-      <c r="J15" s="10" t="inlineStr">
-        <is>
-          <t>Đã chạy tự động bằng Playwright</t>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add test cases for price history (feat/price-history)
Test cases for G3 "Lịch sử giá": every change to selling price or cost
price is logged with who and when, shown on the product page.

- TestCase_3_LichSuGia.docx: 9 test cases (no history yet, price up,
  cost down, other edits add nothing, failed form adds nothing, new
  product starting price, read-only manager, phone layout, cashier has
  no access) with screenshots
- TestCase_SEVEN11.xlsx: new sheet 3-LichSuGia, summary updated
- 8 Pass (7 in a real browser with Playwright on 22/10, 1 by xUnit),
  1 left for manual testing (TC-LSG-09)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/dotnet/docs/test-cases/TestCase_SEVEN11.xlsx
+++ b/apps/dotnet/docs/test-cases/TestCase_SEVEN11.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hồi quy" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1-DoiMatKhau" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2-KhoaDangNhap" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3-LichSuGia" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -530,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -674,31 +675,68 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>3-LichSuGia</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Lịch sử đổi giá bán, giá vốn</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>feat/price-history</t>
+        </is>
+      </c>
+      <c r="D7" s="4">
+        <f>COUNTA('3-LichSuGia'!A5:A13)</f>
+        <v/>
+      </c>
+      <c r="E7" s="4">
+        <f>COUNTIF('3-LichSuGia'!H5:H13,"Pass")</f>
+        <v/>
+      </c>
+      <c r="F7" s="4">
+        <f>COUNTIF('3-LichSuGia'!H5:H13,"Fail")</f>
+        <v/>
+      </c>
+      <c r="G7" s="4">
+        <f>D7-E7-F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="5">
+        <f>IF(D7=0,0,E7/D7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Tổng</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6">
-        <f>SUM(D5:D6)</f>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6">
+        <f>SUM(D5:D7)</f>
         <v/>
       </c>
-      <c r="E7" s="6">
-        <f>SUM(E5:E6)</f>
+      <c r="E8" s="6">
+        <f>SUM(E5:E7)</f>
         <v/>
       </c>
-      <c r="F7" s="6">
-        <f>SUM(F5:F6)</f>
+      <c r="F8" s="6">
+        <f>SUM(F5:F7)</f>
         <v/>
       </c>
-      <c r="G7" s="6">
-        <f>SUM(G5:G6)</f>
+      <c r="G8" s="6">
+        <f>SUM(G5:G7)</f>
         <v/>
       </c>
-      <c r="H7" s="7">
-        <f>IF(D7=0,0,E7/D7)</f>
+      <c r="H8" s="7">
+        <f>IF(D8=0,0,E8/D8)</f>
         <v/>
       </c>
     </row>
@@ -2492,4 +2530,556 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Lịch sử đổi giá bán, giá vốn</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Nhánh: feat/price-history · App .NET: http://localhost:5711 · Tài khoản demo mật khẩu 123456</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Mã TC</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Mục đích kiểm thử</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Điều kiện trước</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Các bước</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Dữ liệu test</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Kết quả mong đợi</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Kết quả thực tế</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Ngày test</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>TC-LSG-01</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Sản phẩm chưa đổi giá lần nào</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập admin@7eleven.demo / 123456</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>1. Sản phẩm → mở một sản phẩm chưa từng đổi giá
+2. Kéo xuống khung Lịch sử giá</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr"/>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Khung Lịch sử giá hiện câu "Chưa đổi giá lần nào…" kèm giá và giá vốn hiện tại</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>TC-LSG-02</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Đổi giá bán</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập admin@7eleven.demo / 123456</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở sản phẩm, tăng giá bán thêm 1.000 ₫
+2. Bấm Lưu thay đổi
+3. Mở lại sản phẩm</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Giá bán: 25.000 → 26.000</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Có 1 dòng: thời gian, người đổi Nguyễn Minh Quân, giá bán 25.000 ₫ → 26.000 ₫ kèm nhãn "Tăng +4%", biên lãi sau khi đổi</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>TC-LSG-03</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Đổi giá vốn</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Đã làm TC-LSG-02</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>1. Giảm giá vốn 500 ₫, bấm Lưu
+2. Mở lại sản phẩm</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Giá vốn: 15.000 → 14.500</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Thêm dòng thứ 2 nằm trên cùng (mới nhất), giá vốn có nhãn "Giảm"</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>TC-LSG-04</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Sửa thông tin khác, không đổi giá</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Đã làm TC-LSG-03</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>1. Sửa thương hiệu, giữ nguyên giá
+2. Bấm Lưu</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr"/>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Lịch sử giá vẫn 2 dòng, không thêm dòng mới</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>TC-LSG-05</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Form bị lỗi thì không ghi lịch sử</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập admin@7eleven.demo / 123456</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhập giá bán 0
+2. Bấm Lưu</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Giá bán: 0</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Báo lỗi "Giá bán phải lớn hơn 0"; lịch sử giá không thêm dòng</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>Kiểm bằng xUnit (PriceHistoryTests)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>TC-LSG-06</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Sản phẩm mới ghi giá ban đầu</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập admin@7eleven.demo / 123456</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Sản phẩm → Thêm sản phẩm, nhập đủ thông tin
+2. Lưu, mở lại sản phẩm vừa thêm</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Giá bán 12.000, giá vốn 8.000</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Lịch sử có 1 dòng ghi "Giá ban đầu" 12.000 ₫</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>TC-LSG-07</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Quản lý cửa hàng chỉ xem</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập quanly1006@7eleven.demo</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở sản phẩm đã đổi giá ở TC-LSG-03</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr"/>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Không có form sửa giá nhưng vẫn thấy đủ lịch sử giá</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>TC-LSG-08</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Hiển thị trên điện thoại</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Trình duyệt ở chế độ điện thoại (390px)</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở sản phẩm có lịch sử giá</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr"/>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Bảng lịch sử cuộn ngang trong khung, cả trang không tràn ngang</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>TC-LSG-09</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Thu ngân không xem được trang sản phẩm</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập thungan1006@7eleven.demo</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Gõ địa chỉ /Admin/Products</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr"/>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Bị chuyển sang trang "Bạn không có quyền xem trang này"</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr"/>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>Chưa test</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr"/>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>Tester chạy tay</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="H5:H13">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H5 H6 H7 H8 H9 H10 H11 H12 H13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pass,Fail,Chưa test"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add test cases for product image upload (feat/product-image-upload)
Test cases for G4 "Tải ảnh sản phẩm": upload JPG/PNG/WEBP up to 2 MB
instead of only pasting a link.

- TestCase_4_AnhSanPham.docx: 13 test cases (wrong type and >2 MB caught
  in the browser, server re-checks size and real file content, preview,
  saved path, new image on product list and storefront, old upload
  deleted on replace, back to a pasted link, phone layout, exactly 2 MB,
  read-only manager) with screenshots
- TestCase_SEVEN11.xlsx: new sheet 4-AnhSanPham; "Hồi quy" adds the
  end-of-day run (xUnit 106/106, Playwright G1-G4 pass)
- 12 Pass (11 in a real browser with Playwright on 22/10, 1 by xUnit),
  1 left for manual testing (TC-ANH-13)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/dotnet/docs/test-cases/TestCase_SEVEN11.xlsx
+++ b/apps/dotnet/docs/test-cases/TestCase_SEVEN11.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1-DoiMatKhau" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2-KhoaDangNhap" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3-LichSuGia" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4-AnhSanPham" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -531,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -712,31 +713,68 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>4-AnhSanPham</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Tải ảnh sản phẩm lên</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>feat/product-image-upload</t>
+        </is>
+      </c>
+      <c r="D8" s="4">
+        <f>COUNTA('4-AnhSanPham'!A5:A17)</f>
+        <v/>
+      </c>
+      <c r="E8" s="4">
+        <f>COUNTIF('4-AnhSanPham'!H5:H17,"Pass")</f>
+        <v/>
+      </c>
+      <c r="F8" s="4">
+        <f>COUNTIF('4-AnhSanPham'!H5:H17,"Fail")</f>
+        <v/>
+      </c>
+      <c r="G8" s="4">
+        <f>D8-E8-F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="5">
+        <f>IF(D8=0,0,E8/D8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Tổng</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6">
-        <f>SUM(D5:D7)</f>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6">
+        <f>SUM(D5:D8)</f>
         <v/>
       </c>
-      <c r="E8" s="6">
-        <f>SUM(E5:E7)</f>
+      <c r="E9" s="6">
+        <f>SUM(E5:E8)</f>
         <v/>
       </c>
-      <c r="F8" s="6">
-        <f>SUM(F5:F7)</f>
+      <c r="F9" s="6">
+        <f>SUM(F5:F8)</f>
         <v/>
       </c>
-      <c r="G8" s="6">
-        <f>SUM(G5:G7)</f>
+      <c r="G9" s="6">
+        <f>SUM(G5:G8)</f>
         <v/>
       </c>
-      <c r="H8" s="7">
-        <f>IF(D8=0,0,E8/D8)</f>
+      <c r="H9" s="7">
+        <f>IF(D9=0,0,E9/D9)</f>
         <v/>
       </c>
     </row>
@@ -751,7 +789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -949,6 +987,83 @@
       <c r="E10" s="8" t="inlineStr">
         <is>
           <t>storefront-flow: nút thêm nhanh ở /khuyen-mai bị ẩn trên điện thoại; có sẵn trên main (bản redesign), cần báo Phát</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Cuối ngày, sau khi làm G3, G4</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>xUnit</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>106/106 đạt</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Cuối ngày, sau khi làm G3, G4</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Playwright G1–G4</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Tạo lại dữ liệu mẫu trước khi chạy</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Cuối ngày, sau khi làm G3, G4</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>e2e của nhóm (admin, pos, storefront-pages, storefront-flow)</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>1 kiểm tra hỏng / 74</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Vẫn là lỗi có sẵn trên main ở trên</t>
         </is>
       </c>
     </row>
@@ -3082,4 +3197,762 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Tải ảnh sản phẩm lên</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Nhánh: feat/product-image-upload · App .NET: http://localhost:5711 · Tài khoản demo mật khẩu 123456</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Mã TC</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Mục đích kiểm thử</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Điều kiện trước</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Các bước</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Dữ liệu test</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Kết quả mong đợi</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Kết quả thực tế</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Ngày test</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>TC-ANH-01</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Form có chỗ tải ảnh</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập admin@7eleven.demo / 123456</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>1. Sản phẩm → mở một sản phẩm</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr"/>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Khung Ảnh sản phẩm có nút "Chọn ảnh từ máy", ô dán đường dẫn và ảnh xem trước</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>TC-ANH-02</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Chọn file sai loại</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở form sản phẩm</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Chọn ảnh từ máy, chọn file .gif</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>anh-dong.gif</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Báo ngay "Chỉ nhận ảnh JPG, PNG hoặc WEBP"</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>TC-ANH-03</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Chọn ảnh quá 2 MB</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở form sản phẩm</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>1. Chọn ảnh JPG 2,9 MB</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>anh-qua-lon.jpg (2,9 MB)</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Báo ngay "Ảnh tối đa 2 MB (file này 2,9 MB)", file bị bỏ chọn</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>TC-ANH-04</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Máy chủ vẫn chặn ảnh quá 2 MB</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Bỏ qua kiểm tra ở trình duyệt</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>1. Chọn ảnh 2,9 MB khi kiểm tra ở trình duyệt bị tắt
+2. Bấm Lưu</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>anh-qua-lon.jpg</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Máy chủ báo "Ảnh tối đa 2 MB (file này 2,9 MB)", không lưu</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>TC-ANH-05</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>File chữ đổi đuôi .jpg</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở form sản phẩm</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Chọn file chữ đặt tên .jpg
+2. Bấm Lưu</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>khong-phai-anh.jpg</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Báo "File không phải ảnh JPG, PNG hoặc WEBP hợp lệ"</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>TC-ANH-06</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Chọn ảnh PNG hợp lệ</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở form sản phẩm</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Chọn ảnh PNG</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>anh-san-pham.png (4 KB)</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Xem trước ngay; hiện tên file và dung lượng; ô đường dẫn cũ bị gạch và khoá</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>TC-ANH-07</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Lưu ảnh tải lên</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Đã làm TC-ANH-06</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Lưu thay đổi
+2. Mở lại sản phẩm</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr"/>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Ảnh lưu thành /uploads/products/&lt;mã&gt;.png, mở được; form ghi "Đang dùng ảnh đã tải lên"</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>TC-ANH-08</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Ảnh mới hiện khắp nơi</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Đã làm TC-ANH-07</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Xem danh sách sản phẩm
+2. Tìm sản phẩm ở cửa hàng online</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr"/>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Danh sách sản phẩm và thẻ sản phẩm ở cửa hàng online dùng ảnh mới</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>TC-ANH-09</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Đổi sang ảnh khác thì ảnh cũ bị xoá</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Đã làm TC-ANH-07</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Chọn ảnh WEBP, Lưu
+2. Mở đường dẫn ảnh PNG cũ</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>anh-san-pham.webp</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Sản phẩm dùng ảnh .webp; ảnh .png cũ trả về 404</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>TC-ANH-10</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Quay lại dán đường dẫn</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Đã làm TC-ANH-09</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. Dán lại link ảnh ban đầu, Lưu</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Link ảnh ban đầu</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Sản phẩm dùng link; ảnh .webp đã tải lên bị dọn (404)</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J14" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>TC-ANH-11</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Hiển thị trên điện thoại</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Trình duyệt ở chế độ điện thoại (390px)</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở form sản phẩm, chọn ảnh JPG</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>anh-san-pham.jpg</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Xem trước và nút chọn ảnh hiển thị đủ, không tràn ngang</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>TC-ANH-12</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Ảnh đúng 2 MB vẫn được nhận</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Có ảnh JPG đúng 2 MB</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. Tải ảnh dung lượng đúng 2 MB</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr"/>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Được nhận; lớn hơn 2 MB 1 byte thì bị từ chối</t>
+        </is>
+      </c>
+      <c r="G16" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="inlineStr">
+        <is>
+          <t>Kiểm bằng xUnit (ProductImagesTests)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>TC-ANH-13</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Quản lý cửa hàng không đổi được ảnh</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập quanly1006@7eleven.demo</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở một sản phẩm</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr"/>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Chỉ xem thông tin, không có form và nút Chọn ảnh từ máy</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="inlineStr"/>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>Chưa test</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="inlineStr"/>
+      <c r="J17" s="12" t="inlineStr">
+        <is>
+          <t>Tester chạy tay</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="H5:H17">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pass,Fail,Chưa test"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add bug notes for the team from testing (LOI-CAN-SUA.md)
Issues found while testing, for Phát to fix:
1. e2e/storefront-flow.cjs hangs when run after the morning flash-sale
   slot: line 331 clicks the first ".pcard .qa-plus" in the HTML, which
   sits in the hidden morning tab. Not a UI bug. Suggested fix
   ".qa-plus:visible", tried on a temp copy: 90/90 pass.
2. e2e results drift across runs: each run places orders for demo
   customer 0901234567 until they reach Diamond, then the "hạng Vàng"
   check fails. Reset demo data in run-all.sh or don't hard-code the tier.
3. README does not say Windows needs only the .NET 8 SDK (the C++ core
   falls back to C#).

Also corrects the "Hồi quy" sheet: the storefront-flow failure was first
logged as a phone-layout issue from the redesign; it is the time-dependent
test above. Adds a row for the 90/90 run with the suggested fix.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/dotnet/docs/test-cases/TestCase_SEVEN11.xlsx
+++ b/apps/dotnet/docs/test-cases/TestCase_SEVEN11.xlsx
@@ -789,7 +789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -986,7 +986,7 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>storefront-flow: nút thêm nhanh ở /khuyen-mai bị ẩn trên điện thoại; có sẵn trên main (bản redesign), cần báo Phát</t>
+          <t>storefront-flow treo: script bấm nút "+" đầu tiên ở /khuyen-mai, nút này nằm trong tab flash sale sáng đang ẩn khi chạy buổi chiều/tối. Lỗi của script trên main, không phải giao diện (xem LOI-CAN-SUA.md, mục 1)</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1063,34 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Vẫn là lỗi có sẵn trên main ở trên</t>
+          <t>Vẫn là lỗi script ở trên (LOI-CAN-SUA.md, mục 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Tối, thử bản sửa gợi ý</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>storefront-flow.cjs với .qa-plus:visible (bản sao tạm, không commit)</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>90/90 đạt</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Xác nhận cách sửa ghi trong LOI-CAN-SUA.md, mục 1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record regression run for G1-G4 on 25/10 and update bug notes
Re-ran every existing test before starting G5/G6 (main had no new
commits):
- xUnit 106/106 pass
- Playwright walk-throughs for G1 change-password, G2 login-lockout,
  G3 price-history, G4 product-image-upload pass (demo data reset first)
- Team e2e: admin-flows, pos-flow, storefront-pages, storefront-flow all
  pass (90/90). storefront-flow passed because it ran at 09:04, inside the
  morning flash-sale slot, which confirms bug 1 in LOI-CAN-SUA.md is
  time-dependent; it is still not fixed on main.

TestCase_SEVEN11.xlsx: G1-G4 rows show the 25/10 run date; "Hồi quy"
sheet gets the 25/10 start-of-day rows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/dotnet/docs/test-cases/TestCase_SEVEN11.xlsx
+++ b/apps/dotnet/docs/test-cases/TestCase_SEVEN11.xlsx
@@ -789,7 +789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1091,6 +1091,83 @@
       <c r="E14" s="8" t="inlineStr">
         <is>
           <t>Xác nhận cách sửa ghi trong LOI-CAN-SUA.md, mục 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Đầu ngày (09:04), main không có commit mới</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>xUnit</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>106/106 đạt</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Đầu ngày (09:04), main không có commit mới</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Playwright G1–G4</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Tạo lại dữ liệu mẫu trước khi chạy</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Đầu ngày (09:04), main không có commit mới</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>e2e của nhóm (admin, pos, storefront-pages, storefront-flow)</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>90/90 đạt</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>storefront-flow đạt vì chạy trong giờ flash sale sáng: khớp phân tích lỗi số 1 (LOI-CAN-SUA.md), lỗi vẫn còn khi chạy chiều/tối</t>
         </is>
       </c>
     </row>
@@ -1231,12 +1308,12 @@
       </c>
       <c r="I5" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J5" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -1279,12 +1356,12 @@
       </c>
       <c r="I6" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1411,12 @@
       </c>
       <c r="I7" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -1387,12 +1464,12 @@
       </c>
       <c r="I8" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -1441,12 +1518,12 @@
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -1495,12 +1572,12 @@
       </c>
       <c r="I10" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J10" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -1549,12 +1626,12 @@
       </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J11" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -1603,12 +1680,12 @@
       </c>
       <c r="I12" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -1652,12 +1729,12 @@
       </c>
       <c r="I13" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J13" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -1704,12 +1781,12 @@
       </c>
       <c r="I14" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J14" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -1757,12 +1834,12 @@
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J15" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -1893,12 +1970,12 @@
       </c>
       <c r="I18" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J18" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -1947,12 +2024,12 @@
       </c>
       <c r="I19" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J19" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -1995,12 +2072,12 @@
       </c>
       <c r="I20" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J20" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -2152,12 +2229,12 @@
       </c>
       <c r="I5" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J5" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -2204,12 +2281,12 @@
       </c>
       <c r="I6" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -2256,12 +2333,12 @@
       </c>
       <c r="I7" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -2308,12 +2385,12 @@
       </c>
       <c r="I8" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -2356,12 +2433,12 @@
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -2405,12 +2482,12 @@
       </c>
       <c r="I10" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J10" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -2455,12 +2532,12 @@
       </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J11" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -2545,12 +2622,12 @@
       </c>
       <c r="I13" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J13" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -2599,12 +2676,12 @@
       </c>
       <c r="I14" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J14" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -2647,12 +2724,12 @@
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J15" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 21/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -2801,12 +2878,12 @@
       </c>
       <c r="I5" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J5" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 22/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -2855,12 +2932,12 @@
       </c>
       <c r="I6" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 22/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -2908,12 +2985,12 @@
       </c>
       <c r="I7" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 22/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -2957,12 +3034,12 @@
       </c>
       <c r="I8" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 22/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -3010,7 +3087,7 @@
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
@@ -3063,12 +3140,12 @@
       </c>
       <c r="I10" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J10" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 22/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -3111,12 +3188,12 @@
       </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J11" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 22/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -3159,12 +3236,12 @@
       </c>
       <c r="I12" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 22/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -3352,12 +3429,12 @@
       </c>
       <c r="I5" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J5" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 22/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -3404,12 +3481,12 @@
       </c>
       <c r="I6" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 22/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -3456,12 +3533,12 @@
       </c>
       <c r="I7" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 22/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -3509,12 +3586,12 @@
       </c>
       <c r="I8" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 22/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -3562,12 +3639,12 @@
       </c>
       <c r="I9" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 22/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -3614,12 +3691,12 @@
       </c>
       <c r="I10" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J10" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 22/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -3663,12 +3740,12 @@
       </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J11" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 22/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -3712,12 +3789,12 @@
       </c>
       <c r="I12" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 22/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -3765,12 +3842,12 @@
       </c>
       <c r="I13" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J13" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 22/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -3817,12 +3894,12 @@
       </c>
       <c r="I14" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J14" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 22/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -3869,12 +3946,12 @@
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J15" s="12" t="inlineStr">
         <is>
-          <t>Chạy tự động bằng Playwright 22/10/2026</t>
+          <t>Chạy tự động bằng Playwright 22/10/2026; chạy lại hồi quy 25/10/2026</t>
         </is>
       </c>
     </row>
@@ -3917,7 +3994,7 @@
       </c>
       <c r="I16" s="12" t="inlineStr">
         <is>
-          <t>22/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="J16" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Add test cases for partial receiving (feat/partial-receiving)
Test cases for G5 "Nhận hàng nhiều đợt": purchase orders received short
over several deliveries, then closed with a reason.

- TestCase_5_NhanHangNhieuDot.docx: 14 test cases (prefilled missing
  quantities, over-receiving and empty delivery refused, first short
  delivery, no cancel once partly received, list progress, second
  delivery, close with reason and billed by received value, nothing more
  after close, full delivery in one go, one lot per delivery, reason
  required, phone layout, dashboard count) with screenshots
- TestCase_SEVEN11.xlsx: new sheet 5-NhanHangNhieuDot, summary updated
- 13 Pass (11 in a real browser with Playwright on 25/10, 2 by xUnit),
  1 left for manual testing (TC-NHD-14)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/dotnet/docs/test-cases/TestCase_SEVEN11.xlsx
+++ b/apps/dotnet/docs/test-cases/TestCase_SEVEN11.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2-KhoaDangNhap" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3-LichSuGia" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4-AnhSanPham" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5-NhanHangNhieuDot" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -532,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -750,31 +751,68 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>5-NhanHangNhieuDot</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Phiếu nhập nhận thiếu, nhận nhiều đợt, kết thúc phiếu</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>feat/partial-receiving</t>
+        </is>
+      </c>
+      <c r="D9" s="4">
+        <f>COUNTA('5-NhanHangNhieuDot'!A5:A18)</f>
+        <v/>
+      </c>
+      <c r="E9" s="4">
+        <f>COUNTIF('5-NhanHangNhieuDot'!H5:H18,"Pass")</f>
+        <v/>
+      </c>
+      <c r="F9" s="4">
+        <f>COUNTIF('5-NhanHangNhieuDot'!H5:H18,"Fail")</f>
+        <v/>
+      </c>
+      <c r="G9" s="4">
+        <f>D9-E9-F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="5">
+        <f>IF(D9=0,0,E9/D9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Tổng</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6">
-        <f>SUM(D5:D8)</f>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6">
+        <f>SUM(D5:D9)</f>
         <v/>
       </c>
-      <c r="E9" s="6">
-        <f>SUM(E5:E8)</f>
+      <c r="E10" s="6">
+        <f>SUM(E5:E9)</f>
         <v/>
       </c>
-      <c r="F9" s="6">
-        <f>SUM(F5:F8)</f>
+      <c r="F10" s="6">
+        <f>SUM(F5:F9)</f>
         <v/>
       </c>
-      <c r="G9" s="6">
-        <f>SUM(G5:G8)</f>
+      <c r="G10" s="6">
+        <f>SUM(G5:G9)</f>
         <v/>
       </c>
-      <c r="H9" s="7">
-        <f>IF(D9=0,0,E9/D9)</f>
+      <c r="H10" s="7">
+        <f>IF(D10=0,0,E10/D10)</f>
         <v/>
       </c>
     </row>
@@ -4059,4 +4097,791 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Phiếu nhập nhận thiếu, nhận nhiều đợt, kết thúc phiếu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Nhánh: feat/partial-receiving · App .NET: http://localhost:5711 · Tài khoản demo mật khẩu 123456</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Mã TC</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Mục đích kiểm thử</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Điều kiện trước</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Các bước</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Dữ liệu test</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Kết quả mong đợi</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Kết quả thực tế</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Ngày test</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>TC-NHD-01</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Phiếu chờ nhận điền sẵn số còn thiếu</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập admin@7eleven.demo / 123456; có phiếu Đã đặt hàng</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhập hàng → lọc Đã đặt hàng → mở một phiếu</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr"/>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Cột "Nhận đợt này" điền sẵn số còn thiếu của từng dòng; còn nút Huỷ phiếu</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>TC-NHD-02</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Không nhận quá số đặt</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở phiếu chờ nhận</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhập ở một dòng số lớn hơn số còn thiếu (bỏ qua giới hạn của trình duyệt)
+2. Bấm Nhận hàng đợt này</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Còn thiếu + 5</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Báo "…chỉ còn thiếu N, không nhận quá số đã đặt"; tồn kho không đổi</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>TC-NHD-03</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Nhận đợt rỗng</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở phiếu chờ nhận</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Đặt tất cả về 0
+2. Bấm Nhận hàng đợt này</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr"/>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Báo "Nhập số lượng nhận cho ít nhất một mặt hàng"</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>TC-NHD-04</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Đợt 1 giao thiếu</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở phiếu chờ nhận</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>1. Đặt tất cả về 0, nhập một nửa ở dòng đầu
+2. Bấm Nhận hàng đợt này</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Dòng đầu: 12/24</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Phiếu sang "Đang nhận hàng"; tồn kho dòng đầu tăng đúng 12; hiện Đã nhận x/y, Còn thiếu, Tiền hàng thực nhận</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>TC-NHD-05</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Phiếu nhận dở không huỷ được</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Đã làm TC-NHD-04</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Xem các nút đầu trang</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr"/>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Không còn nút Huỷ phiếu (chỉ còn Kết thúc phiếu)</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>TC-NHD-06</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Danh sách phiếu hiện tiến độ</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Đã làm TC-NHD-04</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhập hàng → tab Đang nhận hàng</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr"/>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Phiếu nằm ở tab Đang nhận hàng, cột cuối ghi "Đã nhận x/y · hẹn …"</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>TC-NHD-07</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Đợt 2</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Đã làm TC-NHD-04</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhận thêm 1 sản phẩm ở dòng đầu</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr"/>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Khung Các đợt nhận hàng có 2 đợt, mỗi đợt ghi giờ, người nhận, số lượng</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>TC-NHD-08</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Kết thúc phiếu thiếu hàng</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Phiếu đang nhận dở</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở "Kết thúc phiếu", nhập lý do
+2. Bấm Kết thúc phiếu</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Lý do: Nhà cung cấp hết hàng, không giao bù</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Phiếu "Đã kết thúc"; tiền hàng chốt theo số thực nhận; hiện lý do, giờ, người kết thúc</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>TC-NHD-09</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Phiếu đã kết thúc không nhận thêm</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Đã làm TC-NHD-08</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Xem trang phiếu</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr"/>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Không còn cột Nhận đợt này và nút nhận hàng</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>TC-NHD-10</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Giao đủ một lần</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Phiếu Đã đặt hàng khác</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. Bấm Điền đủ phần còn thiếu
+2. Bấm Nhận hàng đợt này</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr"/>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Phiếu "Đã nhập kho", toast "đã nhận đủ và nhập kho xong"</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J14" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>TC-NHD-11</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Hàng có hạn dùng: mỗi đợt một lô</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Phiếu có hàng tươi, nhận 2 đợt</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhận 2 đợt
+2. Xem Lô hàng &amp; hạn dùng</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr"/>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Đợt 1 lô PNxxxxx-SKU, đợt 2 lô PNxxxxx-SKU-D2, hạn tính từ ngày nhận từng đợt</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="inlineStr">
+        <is>
+          <t>Kiểm bằng xUnit (PartialReceivingTests)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>TC-NHD-12</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Kết thúc phiếu phải có lý do</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Phiếu đang nhận dở</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. Kết thúc phiếu với lý do trống</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr"/>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Báo "Nhập lý do kết thúc phiếu…"; phiếu không đổi</t>
+        </is>
+      </c>
+      <c r="G16" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="inlineStr">
+        <is>
+          <t>Kiểm bằng xUnit (PartialReceivingTests)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>TC-NHD-13</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Hiển thị trên điện thoại</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Trình duyệt ở chế độ điện thoại (390px)</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. Nhận một đợt hàng trên điện thoại</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr"/>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Tiến độ, bảng và nút hiển thị đủ; bảng cuộn trong khung, trang không tràn ngang</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>TC-NHD-14</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Tổng quan đếm phiếu nhận dở</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Có phiếu Đang nhận hàng; đăng nhập admin@7eleven.demo / 123456</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở Tổng quan, xem dòng "phiếu nhập chờ nhận hàng"</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr"/>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Phiếu đang nhận dở vẫn được đếm là chờ nhận hàng</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="inlineStr"/>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>Chưa test</t>
+        </is>
+      </c>
+      <c r="I18" s="12" t="inlineStr"/>
+      <c r="J18" s="12" t="inlineStr">
+        <is>
+          <t>Tester chạy tay</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="H5:H18">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pass,Fail,Chưa test"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add test cases for stock transfer (feat/stock-transfer)
Test cases for G6 "Chuyển kho": sender stock goes down on send, receiver
stock goes up on confirm, lots keep their codes and expiry dates.

- TestCase_6_ChuyenKho.docx: 16 test cases (form, expired stock not
  movable, too much refused with entered values kept, send, lots travel
  with perishables, right buttons per side, receiver's waiting count,
  confirm, lot codes and expiry kept, stock log, cancel in transit,
  cashier blocked, phone layout, soonest-expiry lots first, invalid
  destination, admin must pick a store) with screenshots
- TestCase_SEVEN11.xlsx: new sheet 6-ChuyenKho; "Hồi quy" adds the
  end-of-session run (xUnit 117/117, Playwright G1-G6 and team e2e pass)
- 15 Pass (13 in a real browser with Playwright on 25/10, 2 by xUnit),
  1 left for manual testing (TC-CK-16)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/dotnet/docs/test-cases/TestCase_SEVEN11.xlsx
+++ b/apps/dotnet/docs/test-cases/TestCase_SEVEN11.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3-LichSuGia" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4-AnhSanPham" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5-NhanHangNhieuDot" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6-ChuyenKho" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -533,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -788,31 +789,68 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>6-ChuyenKho</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Chuyển kho giữa các cửa hàng</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>feat/stock-transfer</t>
+        </is>
+      </c>
+      <c r="D10" s="4">
+        <f>COUNTA('6-ChuyenKho'!A5:A20)</f>
+        <v/>
+      </c>
+      <c r="E10" s="4">
+        <f>COUNTIF('6-ChuyenKho'!H5:H20,"Pass")</f>
+        <v/>
+      </c>
+      <c r="F10" s="4">
+        <f>COUNTIF('6-ChuyenKho'!H5:H20,"Fail")</f>
+        <v/>
+      </c>
+      <c r="G10" s="4">
+        <f>D10-E10-F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="5">
+        <f>IF(D10=0,0,E10/D10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Tổng</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6">
-        <f>SUM(D5:D9)</f>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6">
+        <f>SUM(D5:D10)</f>
         <v/>
       </c>
-      <c r="E10" s="6">
-        <f>SUM(E5:E9)</f>
+      <c r="E11" s="6">
+        <f>SUM(E5:E10)</f>
         <v/>
       </c>
-      <c r="F10" s="6">
-        <f>SUM(F5:F9)</f>
+      <c r="F11" s="6">
+        <f>SUM(F5:F10)</f>
         <v/>
       </c>
-      <c r="G10" s="6">
-        <f>SUM(G5:G9)</f>
+      <c r="G11" s="6">
+        <f>SUM(G5:G10)</f>
         <v/>
       </c>
-      <c r="H10" s="7">
-        <f>IF(D10=0,0,E10/D10)</f>
+      <c r="H11" s="7">
+        <f>IF(D11=0,0,E11/D11)</f>
         <v/>
       </c>
     </row>
@@ -827,7 +865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1208,6 +1246,79 @@
           <t>storefront-flow đạt vì chạy trong giờ flash sale sáng: khớp phân tích lỗi số 1 (LOI-CAN-SUA.md), lỗi vẫn còn khi chạy chiều/tối</t>
         </is>
       </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Cuối buổi (09:30), sau khi làm G5, G6</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>xUnit</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>117/117 đạt</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Cuối buổi (09:30), sau khi làm G5, G6</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Playwright G1–G6</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Tạo lại dữ liệu mẫu trước khi chạy</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Cuối buổi (09:30), sau khi làm G5, G6</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>e2e của nhóm (admin, pos, storefront-pages, storefront-flow)</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>90/90 đạt</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4884,4 +4995,878 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Chuyển kho giữa các cửa hàng</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Nhánh: feat/stock-transfer · App .NET: http://localhost:5711 · Tài khoản demo mật khẩu 123456</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Mã TC</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Mục đích kiểm thử</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Điều kiện trước</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Các bước</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Dữ liệu test</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Kết quả mong đợi</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Kết quả thực tế</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Ngày test</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>TC-CK-01</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Mở chức năng chuyển kho</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập quanly1006@7eleven.demo</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>1. Menu Hàng hoá → Chuyển kho → Lập phiếu chuyển</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr"/>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Form liệt kê hàng đang có: Tồn hiện có, Chuyển được, Hạn gần nhất, ô số lượng</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>TC-CK-02</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Hàng có hạn dùng đã hết hạn</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Có mặt hàng tươi mà mọi lô đã hết hạn</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>1. Xem dòng mặt hàng đó trong form</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr"/>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Chuyển được = 0, ô nhập bị khoá, dòng mờ và xếp cuối danh sách</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>TC-CK-03</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Chuyển quá số được phép</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở form lập phiếu</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>1. Chọn cửa hàng nhận 1013
+2. Nhập số lớn hơn Chuyển được (bỏ qua giới hạn của trình duyệt)
+3. Bấm Gửi hàng</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Chuyển được + 1</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Báo "…chỉ còn N"; form giữ lại số đã nhập; kho không đổi</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>TC-CK-04</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Gửi hàng</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Đang ở form lập phiếu</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>1. Chọn cửa hàng nhận 1013, nhập 2 hàng tươi + 3 hàng dài hạn, ghi chú
+2. Bấm Gửi hàng</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>2 + 3 sản phẩm</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Tạo phiếu CKxxxxx "Đang chuyển"; kho 1006 trừ ngay đúng số đã gửi</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>TC-CK-05</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Lô đi theo hàng tươi</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Đã làm TC-CK-04</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>1. Xem dòng hàng tươi trên phiếu</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr"/>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Ghi "Lô … × 2 · hạn …"; hàng dài hạn ghi "không theo lô"</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>TC-CK-06</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Đúng người đúng nút</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Đã làm TC-CK-04</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1. Bên gửi xem phiếu
+2. Bên nhận xem phiếu</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr"/>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Bên gửi có Huỷ phiếu, không có Đã nhận hàng; bên nhận ngược lại</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>TC-CK-07</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Bên nhận thấy phiếu chờ</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập quanly1013@7eleven.demo</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>1. Xem menu và tab Chờ nhận</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr"/>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Mục Chuyển kho trên menu có số phiếu chờ; phiếu ghi "chờ bạn nhận"</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>TC-CK-08</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Bên nhận xác nhận</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Đã làm TC-CK-07</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở phiếu, bấm Đã nhận hàng</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr"/>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Phiếu "Đã nhận" (giờ, người nhận); kho 1013 cộng đúng số trên phiếu</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>TC-CK-09</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Giữ nguyên lô và hạn dùng</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Đã làm TC-CK-08</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>1. Kho hàng → Lô hàng &amp; hạn dùng (cửa hàng 1013)</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr"/>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Có lô đúng mã lô ghi trên phiếu, cùng hạn dùng như ở cửa hàng gửi</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>TC-CK-10</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Nhật ký kho</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Đã làm TC-CK-08</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>1. Kho hàng → Nhật ký kho, lọc Nhận chuyển kho, tìm mã phiếu</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr"/>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Có 2 dòng "Nhận chuyển kho" ghi mã phiếu; bên gửi có dòng "Chuyển kho đi"</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J14" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>TC-CK-11</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Huỷ phiếu đang chuyển</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Bên gửi lập thêm phiếu 1 sản phẩm</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở phiếu vừa gửi, bấm Huỷ phiếu</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr"/>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Phiếu "Đã huỷ"; hàng về lại kho bên gửi</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>TC-CK-12</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Thu ngân không dùng được</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập thungan1006@7eleven.demo</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>1. Gõ địa chỉ /Admin/Transfers</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr"/>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Bị chuyển sang trang không có quyền</t>
+        </is>
+      </c>
+      <c r="G16" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>TC-CK-13</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Hiển thị trên điện thoại</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Trình duyệt ở chế độ điện thoại (390px)</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>1. Mở phiếu và form lập phiếu</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr"/>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Không tràn ngang; bảng cuộn trong khung</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="inlineStr">
+        <is>
+          <t>Chạy tự động bằng Playwright 25/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>TC-CK-14</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Lấy lô hết hạn sớm nhất trước, bỏ lô đã hết hạn</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Cửa hàng có lô đã hết hạn, lô 27/10 và lô 30/10</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>1. Chuyển 9 sản phẩm</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr"/>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Lấy hết lô 27/10 rồi 3 từ lô 30/10; lô đã hết hạn giữ nguyên</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I18" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="inlineStr">
+        <is>
+          <t>Kiểm bằng xUnit (StockTransferTests)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>TC-CK-15</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Chặn cửa hàng nhận không hợp lệ</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr"/>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>1. Chuyển tới chính cửa hàng gửi
+2. Chuyển tới cửa hàng đã đóng</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr"/>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Báo "Chọn cửa hàng nhận khác cửa hàng gửi" / "Chọn cửa hàng nhận đang hoạt động"</t>
+        </is>
+      </c>
+      <c r="G19" s="12" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H19" s="12" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="J19" s="12" t="inlineStr">
+        <is>
+          <t>Kiểm bằng xUnit (StockTransferTests)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>TC-CK-16</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Quản trị phải chọn cửa hàng gửi</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Đăng nhập admin@7eleven.demo / 123456, đang xem Toàn chuỗi</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>1. Chuyển kho → Lập phiếu chuyển</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr"/>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Trang nhắc chọn cửa hàng ở ô đầu trang; chọn xong mới lập phiếu được</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr"/>
+      <c r="H20" s="12" t="inlineStr">
+        <is>
+          <t>Chưa test</t>
+        </is>
+      </c>
+      <c r="I20" s="12" t="inlineStr"/>
+      <c r="J20" s="12" t="inlineStr">
+        <is>
+          <t>Tester chạy tay</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="H5:H20">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Pass"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"Fail"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pass,Fail,Chưa test"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>